<commit_message>
Rework ambassador payouts: A monthly+editable, B full rent, C one-time+extra
- Model A: ambassador gets an editable monthly amount (default 200) any month
  the Saudi driver nets >= 5,000; the Saudi driver's own 500/month is now also
  tracked as a company cost.
- Model B: pay the FULL monthly rent to the ambassador (editable, default 500;
  800 for two accounts) instead of the post-split cut; he handles the Saudi
  split privately. Foreigner's incoming rent stays in the Acct/Car Rent IN fields.
- Model C: one-time 500 + editable extra bonus (default 0) at first 6,000 net,
  replacing the fixed +200 support toggle.
- Finance P&L: "Amb." column renamed "Bonuses" = ambassador payout + Model-A
  Saudi 500, with a breakdown line (e.g. "Omar 200 · Saudi 500"); folded into
  netPnL. Profile fields ambAmtA/ambCut/ambExtra replace ambCut/ambSupport.
- Update Bolt_Ambassador_Template (.xlsx/.csv) columns to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bolt_Ambassador_Template.xlsx
+++ b/Bolt_Ambassador_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/205264cd2e922e10/Documents/Claude/Projects/Bolt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{44D9B587-3BA6-4384-AA2E-797D3F6B12E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBB3C705-6FD7-4C29-811F-9C3862B80947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3072" yWindow="840" windowWidth="18096" windowHeight="12840" xr2:uid="{643720C8-B447-4EE9-AF6A-AA27A17CDFE5}"/>
+    <workbookView xWindow="3072" yWindow="840" windowWidth="18096" windowHeight="12840" xr2:uid="{1B9F49B2-4A94-47F7-9A54-2DB6AAB40FFC}"/>
   </bookViews>
   <sheets>
     <sheet name="Bolt_Ambassador_Template" sheetId="1" r:id="rId1"/>
@@ -37,10 +37,13 @@
     <t>1st Trip Date (YYYY-MM-DD)</t>
   </si>
   <si>
-    <t>Model B Cut (SAR)</t>
-  </si>
-  <si>
-    <t>Model C Support (Y/N)</t>
+    <t>Model A monthly amount (SAR)</t>
+  </si>
+  <si>
+    <t>Model B monthly rent (500 or 800)</t>
+  </si>
+  <si>
+    <t>Model C extra bonus (SAR)</t>
   </si>
   <si>
     <t>Notes</t>
@@ -55,7 +58,7 @@
     <t>A</t>
   </si>
   <si>
-    <t>Saudi driver transferred to fleet</t>
+    <t>Saudi driver; Saudi gets 500/mo + Omar 200/mo when net &gt;= 5000</t>
   </si>
   <si>
     <t>ABDULLAH ALQAHTANI</t>
@@ -70,7 +73,7 @@
     <t>B</t>
   </si>
   <si>
-    <t>Saudi user rented to foreigner</t>
+    <t>Two accounts (Bolt+Uber); foreigner rent IN entered in dashboard</t>
   </si>
   <si>
     <t>FAHAD ALOTAIBI</t>
@@ -85,10 +88,7 @@
     <t>C</t>
   </si>
   <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>Existing foreigner + customer support</t>
+    <t>Existing foreigner; one-time 500 + 300 extra at first 6000</t>
   </si>
 </sst>
 </file>
@@ -929,11 +929,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{401C5010-B0DE-458C-9FB6-6054EC32D265}">
-  <dimension ref="A1:H4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E30A2BC-162F-43D6-B285-01E2F033F6BF}">
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -958,61 +958,67 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" t="s">
         <v>11</v>
       </c>
+      <c r="F2">
+        <v>200</v>
+      </c>
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" s="1">
         <v>46162</v>
       </c>
-      <c r="F3">
+      <c r="G3">
+        <v>800</v>
+      </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4">
         <v>300</v>
       </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>